<commit_message>
updating testcase documentation and busaux test descriptions
</commit_message>
<xml_diff>
--- a/Documentation/BusAuxCases with ESS_Formatted.xlsx
+++ b/Documentation/BusAuxCases with ESS_Formatted.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20374"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20375"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C8DCCFE-A7B8-41D1-B4AA-AB582CD2A73B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDFC3F42-173C-4FF8-A5AE-FD8154306743}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="16125" windowHeight="5805" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="16125" windowHeight="5805" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BusAux Case A &amp; Case C2b" sheetId="7" r:id="rId1"/>
@@ -95,15 +95,6 @@
     <t>- P_bat_P0</t>
   </si>
   <si>
-    <t xml:space="preserve"> P_aux_mech</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> P_aux_mech_dr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P_aux_mech </t>
-  </si>
-  <si>
     <t xml:space="preserve"> P_aux_mech_ICEoff_dr</t>
   </si>
   <si>
@@ -128,27 +119,15 @@
     <t>P_PS(n_ice)</t>
   </si>
   <si>
-    <t>P_aux_mech + P_PS(n_ice) + P_ES / AlternatorEfficiency</t>
-  </si>
-  <si>
     <t xml:space="preserve"> P_ES</t>
   </si>
   <si>
     <t xml:space="preserve"> P_ES / AlternatorEfficiency</t>
   </si>
   <si>
-    <t>P_aux_mech + (P_ES - P_ES_ICEOff_dr) / AlternatorEfficiency</t>
-  </si>
-  <si>
-    <t>P_aux_mech + P_PS(n_idle) + P_ES / AlternatorEfficiency</t>
-  </si>
-  <si>
     <t>P_ES / AlternatorEfficiency</t>
   </si>
   <si>
-    <t xml:space="preserve"> P_aux_mech + (P_ES - P_ES_ICEOff_dr) / AlternatorEfficiency</t>
-  </si>
-  <si>
     <t>MaxAlternatorPower - P_ES</t>
   </si>
   <si>
@@ -158,24 +137,12 @@
     <t xml:space="preserve">P_ES - MaxAlternatorPower </t>
   </si>
   <si>
-    <t>P_aux_mech + (P_ES - P_ES_ICEOff_st) / AlternatorEfficiency</t>
-  </si>
-  <si>
     <t>P_ES-MaxAlternatorPower</t>
   </si>
   <si>
     <t>P_aux_mech</t>
   </si>
   <si>
-    <t>P_aux_mech = P_Fan + P_STP + P_PS + P_ES (in case of lorries) + P_HVAC (_mech)</t>
-  </si>
-  <si>
-    <t>P_aux_mech_ICEoff_dr = P_STP + P_PS + P_ES (in case of lorries) + P_HVAC (_mech)</t>
-  </si>
-  <si>
-    <t>P_aux_mech_ICEoff_st = P_PS + P_ES (in case of lorries) + P_HVAC (_mech)</t>
-  </si>
-  <si>
     <t>P_ES = sum of all electric consumers + P_Fan (in case of electric fan) + P_STP (in case of electric steering pump)  -- only used in case of buses</t>
   </si>
   <si>
@@ -236,9 +203,6 @@
     <t xml:space="preserve"> P_ES_ICEOff_st</t>
   </si>
   <si>
-    <t xml:space="preserve"> P_aux_mech + (P_ES - P_ES_ICEOff_st) / AlternatorEfficiency</t>
-  </si>
-  <si>
     <t xml:space="preserve">P_ES = sum of all electric consumers + P_Fan (in case of electric fan) + P_STP (in case of electric steering pump) </t>
   </si>
   <si>
@@ -266,39 +230,6 @@
     <t>P_busAux_ES_consumer_sum</t>
   </si>
   <si>
-    <t xml:space="preserve"> P_aux_mech + P_PS(n_ice)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">			P_aux_mech + P_PS(n_ice) + MaxAlternatorPower / AlternatorEfficiency</t>
-  </si>
-  <si>
-    <t xml:space="preserve">			P_aux_mech + P_PS(n_ice) + P_ES / AlternatorEfficiency</t>
-  </si>
-  <si>
-    <t>P_aux_mech + P_PS(n_ice)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> P_aux_mech + P_PS(n_ice) + MaxAlternatorPower / AlternatorEfficiency</t>
-  </si>
-  <si>
-    <t>P_aux_mech + P_PS(n_ice)+P_ES / AlternatorEff</t>
-  </si>
-  <si>
-    <t>P_aux_mech + P_PS(n_ice) + P_ES / AlternatorEff</t>
-  </si>
-  <si>
-    <t>P_aux_mech + P_PS(n_ice) + MaxAlternatorPower / AlternatorEfficiency</t>
-  </si>
-  <si>
-    <t>P_aux_mech + P_PS(n_idle)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> P_aux_mech + P_PS(n_idle)</t>
-  </si>
-  <si>
-    <t>P_aux_mech + P_PS(n_idle) + P_ES / AlternatorEff</t>
-  </si>
-  <si>
     <t>REESS SoC</t>
   </si>
   <si>
@@ -306,6 +237,75 @@
   </si>
   <si>
     <t>Bus Aux Case C3b: smart alternator, HEV, NO aux supply from REESS</t>
+  </si>
+  <si>
+    <t>P_aux_mech_base + P_PS(n_ice) + P_ES / AlternatorEfficiency</t>
+  </si>
+  <si>
+    <t>P_aux_mech_base + (P_ES - P_ES_ICEOff_dr) / AlternatorEfficiency</t>
+  </si>
+  <si>
+    <t>P_aux_mech_base + P_PS(n_idle) + P_ES / AlternatorEfficiency</t>
+  </si>
+  <si>
+    <t>P_aux_mech_base + (P_ES - P_ES_ICEOff_st) / AlternatorEfficiency</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> P_aux_mech_base + P_PS(n_ice)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> P_aux_mech_base + (P_ES - P_ES_ICEOff_dr) / AlternatorEfficiency</t>
+  </si>
+  <si>
+    <t>P_aux_mech_base + P_PS(n_idle)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> P_aux_mech_base + (P_ES - P_ES_ICEOff_st) / AlternatorEfficiency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">			P_aux_mech_base + P_PS(n_ice) + MaxAlternatorPower / AlternatorEfficiency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">			P_aux_mech_base + P_PS(n_ice) + P_ES / AlternatorEfficiency</t>
+  </si>
+  <si>
+    <t>P_aux_mech_base + P_PS(n_ice)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> P_aux_mech_base</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> P_aux_mech_base_dr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P_aux_mech_base </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> P_aux_mech_base + P_PS(n_idle)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> P_aux_mech_base + P_PS(n_ice) + MaxAlternatorPower / AlternatorEfficiency</t>
+  </si>
+  <si>
+    <t>P_aux_mech_base + P_PS(n_ice)+P_ES / AlternatorEff</t>
+  </si>
+  <si>
+    <t>P_aux_mech_base + P_PS(n_idle) + P_ES / AlternatorEff</t>
+  </si>
+  <si>
+    <t>P_aux_mech_base + P_PS(n_ice) + P_ES / AlternatorEff</t>
+  </si>
+  <si>
+    <t>P_aux_mech_base + P_PS(n_ice) + MaxAlternatorPower / AlternatorEfficiency</t>
+  </si>
+  <si>
+    <t>P_aux_mech_base = P_Fan + P_STP + P_PS (in case of lorries) + P_ES (in case of lorries) + P_HVAC (_mech)</t>
+  </si>
+  <si>
+    <t>P_aux_mech_ICEoff_dr = P_STP + P_PS (in case of lorries) + P_ES (in case of lorries) + P_HVAC (_mech)</t>
+  </si>
+  <si>
+    <t>P_aux_mech_ICEoff_st = P_PS (in case of lorries + P_ES (in case of lorries) + P_HVAC (_mech)</t>
   </si>
 </sst>
 </file>
@@ -1037,21 +1037,21 @@
   <sheetData>
     <row r="1" spans="1:25" s="19" customFormat="1" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A1" s="33" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
     </row>
     <row r="2" spans="1:25" s="19" customFormat="1" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A2" s="33" t="s">
-        <v>65</v>
+        <v>54</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
     </row>
     <row r="3" spans="1:25" s="19" customFormat="1" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A3" s="33" t="s">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
@@ -1091,31 +1091,31 @@
         <v>5</v>
       </c>
       <c r="C5" s="35" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="D5" s="35" t="s">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="E5" s="35" t="s">
-        <v>59</v>
+        <v>48</v>
       </c>
       <c r="F5" s="35" t="s">
         <v>4</v>
       </c>
       <c r="G5" s="35" t="s">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="H5" s="35" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="I5" s="35" t="s">
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="J5" s="35" t="s">
-        <v>63</v>
+        <v>52</v>
       </c>
       <c r="K5" s="36" t="s">
-        <v>64</v>
+        <v>53</v>
       </c>
       <c r="L5" s="37"/>
     </row>
@@ -1127,16 +1127,16 @@
         <v>1</v>
       </c>
       <c r="C6" s="48" t="s">
-        <v>34</v>
+        <v>71</v>
       </c>
       <c r="D6" s="26" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="E6" s="26" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="F6" s="26" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="G6" s="26">
         <v>0</v>
@@ -1151,7 +1151,7 @@
         <v>19</v>
       </c>
       <c r="K6" s="27" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="L6" s="28"/>
     </row>
@@ -1175,10 +1175,10 @@
         <v>0</v>
       </c>
       <c r="G7" s="26" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="H7" s="26" t="s">
-        <v>37</v>
+        <v>72</v>
       </c>
       <c r="I7" s="26">
         <v>0</v>
@@ -1199,16 +1199,16 @@
         <v>1</v>
       </c>
       <c r="C8" s="26" t="s">
-        <v>38</v>
+        <v>73</v>
       </c>
       <c r="D8" s="26" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="E8" s="26" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="F8" s="26" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="G8" s="26">
         <v>0</v>
@@ -1223,7 +1223,7 @@
         <v>19</v>
       </c>
       <c r="K8" s="27" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="L8" s="28"/>
     </row>
@@ -1241,16 +1241,16 @@
         <v>0</v>
       </c>
       <c r="E9" s="26" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="F9" s="26">
         <v>0</v>
       </c>
       <c r="G9" s="26" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="H9" s="26" t="s">
-        <v>44</v>
+        <v>74</v>
       </c>
       <c r="I9" s="26">
         <v>0</v>
@@ -1263,7 +1263,7 @@
       </c>
       <c r="L9" s="28"/>
     </row>
-    <row r="10" spans="1:25" s="1" customFormat="1" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:25" s="1" customFormat="1" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="40" t="s">
         <v>10</v>
       </c>
@@ -1271,16 +1271,16 @@
         <v>1</v>
       </c>
       <c r="C10" s="29" t="s">
-        <v>34</v>
+        <v>71</v>
       </c>
       <c r="D10" s="29" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="E10" s="29" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="F10" s="29" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="G10" s="29">
         <v>0</v>
@@ -1295,7 +1295,7 @@
         <v>19</v>
       </c>
       <c r="K10" s="30" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="L10" s="28"/>
     </row>
@@ -1355,7 +1355,7 @@
     </row>
     <row r="13" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A13" s="23" t="s">
-        <v>47</v>
+        <v>91</v>
       </c>
       <c r="B13" s="24"/>
       <c r="C13" s="24"/>
@@ -1384,7 +1384,7 @@
     </row>
     <row r="14" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A14" s="23" t="s">
-        <v>48</v>
+        <v>92</v>
       </c>
       <c r="B14" s="24"/>
       <c r="C14" s="24"/>
@@ -1413,7 +1413,7 @@
     </row>
     <row r="15" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A15" s="23" t="s">
-        <v>49</v>
+        <v>93</v>
       </c>
       <c r="B15" s="24"/>
       <c r="C15" s="24"/>
@@ -1469,7 +1469,7 @@
     </row>
     <row r="17" spans="1:25" s="19" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="23" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="B17" s="24"/>
       <c r="C17" s="24"/>
@@ -1498,7 +1498,7 @@
     </row>
     <row r="18" spans="1:25" s="19" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="23" t="s">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="B18" s="24"/>
       <c r="C18" s="24"/>
@@ -1527,7 +1527,7 @@
     </row>
     <row r="19" spans="1:25" s="19" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="23" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="B19" s="24"/>
       <c r="C19" s="24"/>
@@ -1583,7 +1583,7 @@
     </row>
     <row r="21" spans="1:25" s="19" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="23" t="s">
-        <v>53</v>
+        <v>42</v>
       </c>
       <c r="B21" s="24"/>
       <c r="C21" s="24"/>
@@ -1612,7 +1612,7 @@
     </row>
     <row r="22" spans="1:25" s="19" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="23" t="s">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="B22" s="24"/>
       <c r="C22" s="24"/>
@@ -1668,7 +1668,7 @@
     </row>
     <row r="24" spans="1:25" s="19" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="23" t="s">
-        <v>55</v>
+        <v>44</v>
       </c>
       <c r="B24" s="24"/>
       <c r="C24" s="24"/>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="25" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A25" s="23" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="B25" s="24"/>
       <c r="C25" s="24"/>
@@ -2653,7 +2653,7 @@
   <sheetData>
     <row r="1" spans="1:25" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A1" s="33" t="s">
-        <v>67</v>
+        <v>56</v>
       </c>
     </row>
     <row r="2" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
@@ -2665,37 +2665,37 @@
         <v>5</v>
       </c>
       <c r="C3" s="54" t="s">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="D3" s="35" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="E3" s="35" t="s">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="F3" s="35" t="s">
         <v>22</v>
       </c>
       <c r="G3" s="35" t="s">
-        <v>59</v>
+        <v>48</v>
       </c>
       <c r="H3" s="35" t="s">
         <v>4</v>
       </c>
       <c r="I3" s="35" t="s">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="J3" s="35" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="K3" s="35" t="s">
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="L3" s="35" t="s">
-        <v>63</v>
+        <v>52</v>
       </c>
       <c r="M3" s="36" t="s">
-        <v>64</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4" spans="1:25" ht="30" x14ac:dyDescent="0.25">
@@ -2709,16 +2709,16 @@
         <v>0.5</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="E4" s="10">
         <v>0</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="H4" s="10">
         <v>0</v>
@@ -2736,7 +2736,7 @@
         <v>19</v>
       </c>
       <c r="M4" s="11" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="N4" s="9"/>
       <c r="O4" s="9"/>
@@ -2762,19 +2762,19 @@
         <v>0</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>34</v>
+        <v>71</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="F5" s="49">
         <v>0</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="I5" s="10">
         <v>0</v>
@@ -2789,7 +2789,7 @@
         <v>19</v>
       </c>
       <c r="M5" s="11" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="N5" s="9"/>
       <c r="O5" s="9"/>
@@ -2830,10 +2830,10 @@
         <v>0</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="J6" s="10" t="s">
-        <v>40</v>
+        <v>76</v>
       </c>
       <c r="K6" s="10">
         <v>0</v>
@@ -2883,10 +2883,10 @@
         <v>0</v>
       </c>
       <c r="I7" s="10" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="J7" s="10" t="s">
-        <v>40</v>
+        <v>76</v>
       </c>
       <c r="K7" s="10">
         <v>0</v>
@@ -2921,16 +2921,16 @@
         <v>0.5</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="E8" s="10">
         <v>0</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="H8" s="10">
         <v>0</v>
@@ -2948,7 +2948,7 @@
         <v>19</v>
       </c>
       <c r="M8" s="11" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="N8" s="9"/>
       <c r="O8" s="9"/>
@@ -2974,19 +2974,19 @@
         <v>0</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>38</v>
+        <v>73</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="F9" s="49">
         <v>0</v>
       </c>
       <c r="G9" s="10" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="H9" s="10" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="I9" s="10">
         <v>0</v>
@@ -3001,7 +3001,7 @@
         <v>19</v>
       </c>
       <c r="M9" s="11" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="N9" s="9"/>
       <c r="O9" s="9"/>
@@ -3033,19 +3033,19 @@
         <v>0</v>
       </c>
       <c r="F10" s="10" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="H10" s="10">
         <v>0</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="J10" s="10" t="s">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="K10" s="10">
         <v>0</v>
@@ -3089,16 +3089,16 @@
         <v>0</v>
       </c>
       <c r="G11" s="10" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="H11" s="10">
         <v>0</v>
       </c>
       <c r="I11" s="10" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="J11" s="10" t="s">
-        <v>44</v>
+        <v>74</v>
       </c>
       <c r="K11" s="10">
         <v>0</v>
@@ -3133,16 +3133,16 @@
         <v>0.5</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="E12" s="10" t="s">
         <v>8</v>
       </c>
       <c r="F12" s="49" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="H12" s="10" t="s">
         <v>9</v>
@@ -3160,7 +3160,7 @@
         <v>19</v>
       </c>
       <c r="M12" s="11" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="N12" s="9"/>
       <c r="O12" s="9"/>
@@ -3186,19 +3186,19 @@
         <v>1</v>
       </c>
       <c r="D13" s="12" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="E13" s="12" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="F13" s="53">
         <v>0</v>
       </c>
       <c r="G13" s="12" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="H13" s="12" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="I13" s="12">
         <v>0</v>
@@ -3213,7 +3213,7 @@
         <v>19</v>
       </c>
       <c r="M13" s="13" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="N13" s="9"/>
       <c r="O13" s="9"/>
@@ -3229,18 +3229,18 @@
       <c r="Y13" s="9"/>
     </row>
     <row r="16" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A16" s="46" t="s">
-        <v>47</v>
+      <c r="A16" s="23" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="46" t="s">
-        <v>48</v>
+      <c r="A17" s="23" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="46" t="s">
-        <v>49</v>
+      <c r="A18" s="23" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
@@ -3248,12 +3248,12 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="46" t="s">
-        <v>71</v>
+        <v>59</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A21" s="46" t="s">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="B21" s="44"/>
       <c r="C21" s="44"/>
@@ -3262,7 +3262,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="46" t="s">
-        <v>73</v>
+        <v>61</v>
       </c>
       <c r="E22" s="45"/>
     </row>
@@ -3272,13 +3272,13 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="46" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="E24" s="45"/>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="46" t="s">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="E25" s="45"/>
     </row>
@@ -3288,13 +3288,13 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="46" t="s">
-        <v>55</v>
+        <v>44</v>
       </c>
       <c r="E27" s="45"/>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="46" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="E28" s="45"/>
     </row>
@@ -3380,12 +3380,12 @@
   <sheetData>
     <row r="1" spans="1:15" s="19" customFormat="1" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A1" s="33" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2" spans="1:15" s="19" customFormat="1" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A2" s="33" t="s">
-        <v>76</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
@@ -3400,40 +3400,40 @@
         <v>21</v>
       </c>
       <c r="D4" s="35" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="E4" s="35" t="s">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="F4" s="35" t="s">
         <v>22</v>
       </c>
       <c r="G4" s="35" t="s">
-        <v>79</v>
+        <v>67</v>
       </c>
       <c r="H4" s="35" t="s">
         <v>4</v>
       </c>
       <c r="I4" s="35" t="s">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="J4" s="35" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="K4" s="35" t="s">
-        <v>77</v>
+        <v>65</v>
       </c>
       <c r="L4" s="35" t="s">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="M4" s="35" t="s">
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="N4" s="35" t="s">
-        <v>63</v>
+        <v>52</v>
       </c>
       <c r="O4" s="36" t="s">
-        <v>64</v>
+        <v>53</v>
       </c>
     </row>
     <row r="5" spans="1:15" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -3447,7 +3447,7 @@
         <v>0.5</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="E5" s="10">
         <v>0</v>
@@ -3456,7 +3456,7 @@
         <v>0</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="H5" s="10">
         <v>0</v>
@@ -3468,7 +3468,7 @@
         <v>0</v>
       </c>
       <c r="K5" s="10" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="L5" s="10">
         <v>0</v>
@@ -3480,7 +3480,7 @@
         <v>19</v>
       </c>
       <c r="O5" s="11" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:15" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -3494,7 +3494,7 @@
         <v>12</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="E6" s="10">
         <v>0</v>
@@ -3503,7 +3503,7 @@
         <v>0</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="H6" s="10">
         <v>0</v>
@@ -3518,7 +3518,7 @@
         <v>0</v>
       </c>
       <c r="L6" s="10" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="M6" s="10" t="s">
         <v>19</v>
@@ -3527,7 +3527,7 @@
         <v>19</v>
       </c>
       <c r="O6" s="11" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:15" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -3556,10 +3556,10 @@
         <v>0</v>
       </c>
       <c r="I7" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="J7" s="10" t="s">
-        <v>23</v>
+        <v>82</v>
       </c>
       <c r="K7" s="10" t="s">
         <v>3</v>
@@ -3603,10 +3603,10 @@
         <v>0</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="J8" s="10" t="s">
-        <v>24</v>
+        <v>83</v>
       </c>
       <c r="K8" s="10">
         <v>0</v>
@@ -3635,7 +3635,7 @@
         <v>0.5</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="E9" s="10">
         <v>0</v>
@@ -3644,7 +3644,7 @@
         <v>0</v>
       </c>
       <c r="G9" s="10" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="H9" s="10">
         <v>0</v>
@@ -3656,7 +3656,7 @@
         <v>0</v>
       </c>
       <c r="K9" s="10" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="L9" s="10">
         <v>0</v>
@@ -3668,7 +3668,7 @@
         <v>19</v>
       </c>
       <c r="O9" s="11" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="10" spans="1:15" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -3682,7 +3682,7 @@
         <v>12</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="E10" s="10">
         <v>0</v>
@@ -3691,7 +3691,7 @@
         <v>0</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="H10" s="10">
         <v>0</v>
@@ -3706,7 +3706,7 @@
         <v>0</v>
       </c>
       <c r="L10" s="10" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="M10" s="10" t="s">
         <v>19</v>
@@ -3715,7 +3715,7 @@
         <v>19</v>
       </c>
       <c r="O10" s="11" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="11" spans="1:15" s="9" customFormat="1" x14ac:dyDescent="0.25">
@@ -3738,19 +3738,19 @@
         <v>0</v>
       </c>
       <c r="G11" s="10" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="H11" s="10">
         <v>0</v>
       </c>
       <c r="I11" s="10" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="J11" s="10" t="s">
-        <v>23</v>
+        <v>82</v>
       </c>
       <c r="K11" s="10" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="L11" s="10">
         <v>0</v>
@@ -3785,22 +3785,22 @@
         <v>0</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="H12" s="10">
         <v>0</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="J12" s="10" t="s">
-        <v>23</v>
+        <v>82</v>
       </c>
       <c r="K12" s="10">
         <v>0</v>
       </c>
       <c r="L12" s="10" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="M12" s="10">
         <v>0</v>
@@ -3823,7 +3823,7 @@
         <v>0.5</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="E13" s="10">
         <v>0</v>
@@ -3832,7 +3832,7 @@
         <v>0</v>
       </c>
       <c r="G13" s="10" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="H13" s="10">
         <v>0</v>
@@ -3844,7 +3844,7 @@
         <v>0</v>
       </c>
       <c r="K13" s="10" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="L13" s="10">
         <v>0</v>
@@ -3856,7 +3856,7 @@
         <v>19</v>
       </c>
       <c r="O13" s="11" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="14" spans="1:15" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -3870,7 +3870,7 @@
         <v>12</v>
       </c>
       <c r="D14" s="10" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="E14" s="10">
         <v>0</v>
@@ -3879,7 +3879,7 @@
         <v>0</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="H14" s="10">
         <v>0</v>
@@ -3894,7 +3894,7 @@
         <v>0</v>
       </c>
       <c r="L14" s="10" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="M14" s="10" t="s">
         <v>19</v>
@@ -3903,7 +3903,7 @@
         <v>19</v>
       </c>
       <c r="O14" s="11" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="15" spans="1:15" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -3932,10 +3932,10 @@
         <v>0</v>
       </c>
       <c r="I15" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="J15" s="10" t="s">
-        <v>23</v>
+        <v>82</v>
       </c>
       <c r="K15" s="10" t="s">
         <v>3</v>
@@ -3979,10 +3979,10 @@
         <v>0</v>
       </c>
       <c r="I16" s="12" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="J16" s="12" t="s">
-        <v>23</v>
+        <v>82</v>
       </c>
       <c r="K16" s="12">
         <v>0</v>
@@ -4001,18 +4001,18 @@
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="46" t="s">
-        <v>47</v>
+      <c r="A19" s="23" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="46" t="s">
-        <v>48</v>
+      <c r="A20" s="23" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="46" t="s">
-        <v>49</v>
+      <c r="A21" s="23" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
@@ -4020,12 +4020,12 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="46" t="s">
-        <v>71</v>
+        <v>59</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="46" t="s">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="B24" s="7"/>
       <c r="C24" s="7"/>
@@ -4033,7 +4033,7 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="46" t="s">
-        <v>73</v>
+        <v>61</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
@@ -4041,12 +4041,12 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="46" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="46" t="s">
-        <v>54</v>
+        <v>43</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
@@ -4054,12 +4054,12 @@
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="46" t="s">
-        <v>55</v>
+        <v>44</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="46" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -4095,7 +4095,7 @@
   <sheetData>
     <row r="1" spans="1:17" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A1" s="33" t="s">
-        <v>92</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
@@ -4107,49 +4107,49 @@
         <v>14</v>
       </c>
       <c r="C3" s="35" t="s">
+        <v>57</v>
+      </c>
+      <c r="D3" s="35" t="s">
         <v>68</v>
-      </c>
-      <c r="D3" s="35" t="s">
-        <v>91</v>
       </c>
       <c r="E3" s="35" t="s">
         <v>16</v>
       </c>
       <c r="F3" s="35" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="G3" s="35" t="s">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="H3" s="35" t="s">
         <v>22</v>
       </c>
       <c r="I3" s="35" t="s">
-        <v>79</v>
+        <v>67</v>
       </c>
       <c r="J3" s="35" t="s">
         <v>4</v>
       </c>
       <c r="K3" s="35" t="s">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="L3" s="35" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="M3" s="35" t="s">
-        <v>77</v>
+        <v>65</v>
       </c>
       <c r="N3" s="35" t="s">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="O3" s="35" t="s">
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="P3" s="35" t="s">
-        <v>63</v>
+        <v>52</v>
       </c>
       <c r="Q3" s="36" t="s">
-        <v>64</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
@@ -4169,16 +4169,16 @@
         <v>0</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="G4" s="10">
         <v>0</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="J4" s="10">
         <v>0</v>
@@ -4202,7 +4202,7 @@
         <v>19</v>
       </c>
       <c r="Q4" s="11" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
@@ -4222,7 +4222,7 @@
         <v>0</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="G5" s="10">
         <v>0</v>
@@ -4231,7 +4231,7 @@
         <v>0</v>
       </c>
       <c r="I5" s="10" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="J5" s="10">
         <v>0</v>
@@ -4243,7 +4243,7 @@
         <v>0</v>
       </c>
       <c r="M5" s="10" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="N5" s="10">
         <v>0</v>
@@ -4255,7 +4255,7 @@
         <v>19</v>
       </c>
       <c r="Q5" s="11" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
@@ -4275,16 +4275,16 @@
         <v>0</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="G6" s="10">
         <v>0</v>
       </c>
       <c r="H6" s="10" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="J6" s="10">
         <v>0</v>
@@ -4308,7 +4308,7 @@
         <v>19</v>
       </c>
       <c r="Q6" s="11" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
@@ -4328,7 +4328,7 @@
         <v>0</v>
       </c>
       <c r="F7" s="10" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="G7" s="10">
         <v>0</v>
@@ -4337,7 +4337,7 @@
         <v>0</v>
       </c>
       <c r="I7" s="10" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="J7" s="10">
         <v>0</v>
@@ -4352,7 +4352,7 @@
         <v>0</v>
       </c>
       <c r="N7" s="10" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="O7" s="10" t="s">
         <v>19</v>
@@ -4361,7 +4361,7 @@
         <v>19</v>
       </c>
       <c r="Q7" s="11" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
@@ -4415,10 +4415,10 @@
         <v>0</v>
       </c>
       <c r="K9" s="10" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="L9" s="10" t="s">
-        <v>25</v>
+        <v>84</v>
       </c>
       <c r="M9" s="10">
         <v>0</v>
@@ -4468,10 +4468,10 @@
         <v>0</v>
       </c>
       <c r="K10" s="10" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="L10" s="10" t="s">
-        <v>25</v>
+        <v>84</v>
       </c>
       <c r="M10" s="10" t="s">
         <v>13</v>
@@ -4521,10 +4521,10 @@
         <v>0</v>
       </c>
       <c r="K11" s="10" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="L11" s="10" t="s">
-        <v>25</v>
+        <v>84</v>
       </c>
       <c r="M11" s="10">
         <v>0</v>
@@ -4574,10 +4574,10 @@
         <v>0</v>
       </c>
       <c r="K12" s="10" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="L12" s="10" t="s">
-        <v>25</v>
+        <v>84</v>
       </c>
       <c r="M12" s="10">
         <v>0</v>
@@ -4631,16 +4631,16 @@
         <v>0</v>
       </c>
       <c r="F14" s="10" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="G14" s="10">
         <v>0</v>
       </c>
       <c r="H14" s="10" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="J14" s="10">
         <v>0</v>
@@ -4664,7 +4664,7 @@
         <v>19</v>
       </c>
       <c r="Q14" s="11" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.25">
@@ -4684,7 +4684,7 @@
         <v>0</v>
       </c>
       <c r="F15" s="10" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="G15" s="10">
         <v>0</v>
@@ -4693,7 +4693,7 @@
         <v>0</v>
       </c>
       <c r="I15" s="10" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="J15" s="10">
         <v>0</v>
@@ -4705,7 +4705,7 @@
         <v>0</v>
       </c>
       <c r="M15" s="10" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="N15" s="10">
         <v>0</v>
@@ -4717,7 +4717,7 @@
         <v>19</v>
       </c>
       <c r="Q15" s="11" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.25">
@@ -4737,16 +4737,16 @@
         <v>0</v>
       </c>
       <c r="F16" s="10" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="G16" s="10">
         <v>0</v>
       </c>
       <c r="H16" s="10" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="J16" s="10">
         <v>0</v>
@@ -4770,7 +4770,7 @@
         <v>19</v>
       </c>
       <c r="Q16" s="11" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="17" spans="1:17" x14ac:dyDescent="0.25">
@@ -4790,7 +4790,7 @@
         <v>0</v>
       </c>
       <c r="F17" s="10" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="G17" s="10">
         <v>0</v>
@@ -4799,7 +4799,7 @@
         <v>0</v>
       </c>
       <c r="I17" s="10" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="J17" s="10">
         <v>0</v>
@@ -4814,7 +4814,7 @@
         <v>0</v>
       </c>
       <c r="N17" s="10" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="O17" s="10" t="s">
         <v>19</v>
@@ -4823,7 +4823,7 @@
         <v>19</v>
       </c>
       <c r="Q17" s="11" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="18" spans="1:17" x14ac:dyDescent="0.25">
@@ -4877,10 +4877,10 @@
         <v>0</v>
       </c>
       <c r="K19" s="10" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="L19" s="10" t="s">
-        <v>25</v>
+        <v>84</v>
       </c>
       <c r="M19" s="10">
         <v>0</v>
@@ -4930,10 +4930,10 @@
         <v>0</v>
       </c>
       <c r="K20" s="10" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="L20" s="10" t="s">
-        <v>25</v>
+        <v>84</v>
       </c>
       <c r="M20" s="10" t="s">
         <v>17</v>
@@ -4983,10 +4983,10 @@
         <v>0</v>
       </c>
       <c r="K21" s="10" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="L21" s="10" t="s">
-        <v>25</v>
+        <v>84</v>
       </c>
       <c r="M21" s="10">
         <v>0</v>
@@ -5036,10 +5036,10 @@
         <v>0</v>
       </c>
       <c r="K22" s="10" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="L22" s="10" t="s">
-        <v>25</v>
+        <v>84</v>
       </c>
       <c r="M22" s="10">
         <v>0</v>
@@ -5093,16 +5093,16 @@
         <v>0.5</v>
       </c>
       <c r="F24" s="10" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="G24" s="10">
         <v>0</v>
       </c>
       <c r="H24" s="10" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="I24" s="10" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="J24" s="10">
         <v>0</v>
@@ -5126,7 +5126,7 @@
         <v>19</v>
       </c>
       <c r="Q24" s="11" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="25" spans="1:17" x14ac:dyDescent="0.25">
@@ -5146,7 +5146,7 @@
         <v>0.5</v>
       </c>
       <c r="F25" s="10" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="G25" s="10">
         <v>0</v>
@@ -5155,7 +5155,7 @@
         <v>0</v>
       </c>
       <c r="I25" s="10" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="J25" s="10">
         <v>0</v>
@@ -5167,7 +5167,7 @@
         <v>0</v>
       </c>
       <c r="M25" s="10" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="N25" s="10">
         <v>0</v>
@@ -5179,7 +5179,7 @@
         <v>19</v>
       </c>
       <c r="Q25" s="11" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="26" spans="1:17" x14ac:dyDescent="0.25">
@@ -5199,16 +5199,16 @@
         <v>0.5</v>
       </c>
       <c r="F26" s="10" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="G26" s="10">
         <v>0</v>
       </c>
       <c r="H26" s="10" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="I26" s="10" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="J26" s="10">
         <v>0</v>
@@ -5232,7 +5232,7 @@
         <v>19</v>
       </c>
       <c r="Q26" s="11" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="27" spans="1:17" x14ac:dyDescent="0.25">
@@ -5252,7 +5252,7 @@
         <v>0.5</v>
       </c>
       <c r="F27" s="10" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="G27" s="10">
         <v>0</v>
@@ -5261,7 +5261,7 @@
         <v>0</v>
       </c>
       <c r="I27" s="10" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="J27" s="10">
         <v>0</v>
@@ -5276,7 +5276,7 @@
         <v>0</v>
       </c>
       <c r="N27" s="10" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="O27" s="10" t="s">
         <v>19</v>
@@ -5285,7 +5285,7 @@
         <v>19</v>
       </c>
       <c r="Q27" s="11" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="28" spans="1:17" x14ac:dyDescent="0.25">
@@ -5339,10 +5339,10 @@
         <v>0</v>
       </c>
       <c r="K29" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="L29" s="10" t="s">
-        <v>25</v>
+        <v>84</v>
       </c>
       <c r="M29" s="10">
         <v>0</v>
@@ -5392,10 +5392,10 @@
         <v>0</v>
       </c>
       <c r="K30" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="L30" s="10" t="s">
-        <v>25</v>
+        <v>84</v>
       </c>
       <c r="M30" s="10" t="s">
         <v>13</v>
@@ -5445,10 +5445,10 @@
         <v>0</v>
       </c>
       <c r="K31" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="L31" s="10" t="s">
-        <v>25</v>
+        <v>84</v>
       </c>
       <c r="M31" s="10">
         <v>0</v>
@@ -5498,10 +5498,10 @@
         <v>0</v>
       </c>
       <c r="K32" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="L32" s="10" t="s">
-        <v>25</v>
+        <v>84</v>
       </c>
       <c r="M32" s="10">
         <v>0</v>
@@ -5555,16 +5555,16 @@
         <v>1</v>
       </c>
       <c r="F34" s="10" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G34" s="10" t="s">
         <v>15</v>
       </c>
       <c r="H34" s="10" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="I34" s="10" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="J34" s="10" t="s">
         <v>18</v>
@@ -5588,7 +5588,7 @@
         <v>19</v>
       </c>
       <c r="Q34" s="11" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="35" spans="1:17" ht="45" x14ac:dyDescent="0.25">
@@ -5608,16 +5608,16 @@
         <v>1</v>
       </c>
       <c r="F35" s="10" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G35" s="10" t="s">
         <v>15</v>
       </c>
       <c r="H35" s="10" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="I35" s="10" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="J35" s="10" t="s">
         <v>18</v>
@@ -5641,7 +5641,7 @@
         <v>19</v>
       </c>
       <c r="Q35" s="11" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="36" spans="1:17" ht="45" x14ac:dyDescent="0.25">
@@ -5661,16 +5661,16 @@
         <v>1</v>
       </c>
       <c r="F36" s="10" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G36" s="10" t="s">
         <v>15</v>
       </c>
       <c r="H36" s="10" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="I36" s="10" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="J36" s="10" t="s">
         <v>18</v>
@@ -5694,7 +5694,7 @@
         <v>19</v>
       </c>
       <c r="Q36" s="11" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="37" spans="1:17" ht="45" x14ac:dyDescent="0.25">
@@ -5714,16 +5714,16 @@
         <v>1</v>
       </c>
       <c r="F37" s="10" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G37" s="10" t="s">
         <v>15</v>
       </c>
       <c r="H37" s="10" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="I37" s="10" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="J37" s="10" t="s">
         <v>18</v>
@@ -5747,7 +5747,7 @@
         <v>19</v>
       </c>
       <c r="Q37" s="11" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="38" spans="1:17" x14ac:dyDescent="0.25">
@@ -5801,10 +5801,10 @@
         <v>0</v>
       </c>
       <c r="K39" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="L39" s="10" t="s">
-        <v>25</v>
+        <v>84</v>
       </c>
       <c r="M39" s="10">
         <v>0</v>
@@ -5854,10 +5854,10 @@
         <v>0</v>
       </c>
       <c r="K40" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="L40" s="10" t="s">
-        <v>25</v>
+        <v>84</v>
       </c>
       <c r="M40" s="10" t="s">
         <v>13</v>
@@ -5907,10 +5907,10 @@
         <v>0</v>
       </c>
       <c r="K41" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="L41" s="10" t="s">
-        <v>25</v>
+        <v>84</v>
       </c>
       <c r="M41" s="10">
         <v>0</v>
@@ -5960,10 +5960,10 @@
         <v>0</v>
       </c>
       <c r="K42" s="12" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="L42" s="12" t="s">
-        <v>25</v>
+        <v>84</v>
       </c>
       <c r="M42" s="12">
         <v>0</v>
@@ -5982,13 +5982,13 @@
       </c>
     </row>
     <row r="45" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A45" s="46" t="s">
-        <v>47</v>
+      <c r="A45" s="23" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="46" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A46" s="46" t="s">
-        <v>48</v>
+      <c r="A46" s="23" t="s">
+        <v>92</v>
       </c>
       <c r="B46" s="7"/>
       <c r="C46" s="7"/>
@@ -5996,8 +5996,8 @@
       <c r="E46" s="7"/>
     </row>
     <row r="47" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A47" s="46" t="s">
-        <v>49</v>
+      <c r="A47" s="23" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="48" spans="1:17" x14ac:dyDescent="0.25">
@@ -6005,17 +6005,17 @@
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" s="46" t="s">
-        <v>71</v>
+        <v>59</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" s="46" t="s">
-        <v>72</v>
+        <v>60</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" s="46" t="s">
-        <v>73</v>
+        <v>61</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
@@ -6023,12 +6023,12 @@
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" s="46" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" s="46" t="s">
-        <v>54</v>
+        <v>43</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.25">
@@ -6036,12 +6036,12 @@
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A56" s="46" t="s">
-        <v>55</v>
+        <v>44</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" s="46" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -6073,7 +6073,7 @@
   <sheetData>
     <row r="1" spans="1:14" s="19" customFormat="1" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A1" s="33" t="s">
-        <v>93</v>
+        <v>70</v>
       </c>
       <c r="K1" s="15"/>
       <c r="L1" s="15"/>
@@ -6094,40 +6094,40 @@
         <v>14</v>
       </c>
       <c r="C3" s="35" t="s">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="D3" s="35" t="s">
         <v>16</v>
       </c>
       <c r="E3" s="35" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="F3" s="35" t="s">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="G3" s="35" t="s">
         <v>22</v>
       </c>
       <c r="H3" s="35" t="s">
-        <v>79</v>
+        <v>67</v>
       </c>
       <c r="I3" s="35" t="s">
         <v>4</v>
       </c>
       <c r="J3" s="35" t="s">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="K3" s="35" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="L3" s="35" t="s">
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="M3" s="35" t="s">
-        <v>63</v>
+        <v>52</v>
       </c>
       <c r="N3" s="36" t="s">
-        <v>64</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
@@ -6144,16 +6144,16 @@
         <v>0</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="F4" s="10">
         <v>0</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="I4" s="10">
         <v>0</v>
@@ -6171,7 +6171,7 @@
         <v>19</v>
       </c>
       <c r="N4" s="11" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:14" ht="45" x14ac:dyDescent="0.25">
@@ -6188,19 +6188,19 @@
         <v>0</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="G5" s="10">
         <v>0</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="I5" s="10" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="J5" s="10">
         <v>0</v>
@@ -6215,7 +6215,7 @@
         <v>19</v>
       </c>
       <c r="N5" s="11" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:14" ht="45" x14ac:dyDescent="0.25">
@@ -6247,10 +6247,10 @@
         <v>0</v>
       </c>
       <c r="J6" s="10" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="K6" s="10" t="s">
-        <v>37</v>
+        <v>72</v>
       </c>
       <c r="L6" s="10">
         <v>0</v>
@@ -6291,10 +6291,10 @@
         <v>0</v>
       </c>
       <c r="J7" s="10" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="K7" s="10" t="s">
-        <v>37</v>
+        <v>72</v>
       </c>
       <c r="L7" s="10">
         <v>0</v>
@@ -6336,16 +6336,16 @@
         <v>0</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="F9" s="10">
         <v>0</v>
       </c>
       <c r="G9" s="10" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="H9" s="10" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="I9" s="10">
         <v>0</v>
@@ -6363,7 +6363,7 @@
         <v>19</v>
       </c>
       <c r="N9" s="11" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="30" x14ac:dyDescent="0.25">
@@ -6380,19 +6380,19 @@
         <v>0</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="F10" s="10" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="G10" s="10">
         <v>0</v>
       </c>
       <c r="H10" s="10" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="J10" s="10">
         <v>0</v>
@@ -6407,7 +6407,7 @@
         <v>19</v>
       </c>
       <c r="N10" s="11" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="11" spans="1:14" ht="45" x14ac:dyDescent="0.25">
@@ -6439,10 +6439,10 @@
         <v>0</v>
       </c>
       <c r="J11" s="10" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="K11" s="10" t="s">
-        <v>44</v>
+        <v>74</v>
       </c>
       <c r="L11" s="10">
         <v>0</v>
@@ -6483,10 +6483,10 @@
         <v>0</v>
       </c>
       <c r="J12" s="10" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="K12" s="10" t="s">
-        <v>44</v>
+        <v>74</v>
       </c>
       <c r="L12" s="10">
         <v>0</v>
@@ -6528,16 +6528,16 @@
         <v>0.5</v>
       </c>
       <c r="E14" s="55" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="F14" s="55">
         <v>0</v>
       </c>
       <c r="G14" s="55" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="H14" s="55" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="I14" s="55">
         <v>0</v>
@@ -6555,7 +6555,7 @@
         <v>19</v>
       </c>
       <c r="N14" s="11" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
@@ -6572,16 +6572,16 @@
         <v>0.5</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="F15" s="55">
         <v>0</v>
       </c>
       <c r="G15" s="10" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="H15" s="55" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="I15" s="10">
         <v>0</v>
@@ -6599,7 +6599,7 @@
         <v>19</v>
       </c>
       <c r="N15" s="11" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="16" spans="1:14" s="8" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -6616,19 +6616,19 @@
         <v>0.5</v>
       </c>
       <c r="E16" s="55" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="F16" s="55" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="G16" s="55">
         <v>0</v>
       </c>
       <c r="H16" s="55" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="J16" s="55">
         <v>0</v>
@@ -6643,7 +6643,7 @@
         <v>19</v>
       </c>
       <c r="N16" s="11" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="17" spans="1:14" ht="45" x14ac:dyDescent="0.25">
@@ -6675,10 +6675,10 @@
         <v>0</v>
       </c>
       <c r="J17" s="55" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="K17" s="10" t="s">
-        <v>37</v>
+        <v>72</v>
       </c>
       <c r="L17" s="10">
         <v>0</v>
@@ -6719,10 +6719,10 @@
         <v>0</v>
       </c>
       <c r="J18" s="55" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="K18" s="10" t="s">
-        <v>37</v>
+        <v>72</v>
       </c>
       <c r="L18" s="10">
         <v>0</v>
@@ -6763,10 +6763,10 @@
         <v>0</v>
       </c>
       <c r="J19" s="55" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="K19" s="10" t="s">
-        <v>37</v>
+        <v>72</v>
       </c>
       <c r="L19" s="10">
         <v>0</v>
@@ -6808,16 +6808,16 @@
         <v>1</v>
       </c>
       <c r="E21" s="55" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="F21" s="55" t="s">
         <v>15</v>
       </c>
       <c r="G21" s="55" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="H21" s="55" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="I21" s="55" t="s">
         <v>18</v>
@@ -6835,7 +6835,7 @@
         <v>19</v>
       </c>
       <c r="N21" s="11" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="22" spans="1:14" ht="30" x14ac:dyDescent="0.25">
@@ -6852,19 +6852,19 @@
         <v>1</v>
       </c>
       <c r="E22" s="55" t="s">
-        <v>34</v>
+        <v>71</v>
       </c>
       <c r="F22" s="55" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="G22" s="55">
         <v>0</v>
       </c>
       <c r="H22" s="55" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="I22" s="55" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="J22" s="55">
         <v>0</v>
@@ -6879,7 +6879,7 @@
         <v>19</v>
       </c>
       <c r="N22" s="11" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="23" spans="1:14" s="8" customFormat="1" ht="45" x14ac:dyDescent="0.25">
@@ -6896,16 +6896,16 @@
         <v>1</v>
       </c>
       <c r="E23" s="55" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="F23" s="55" t="s">
         <v>15</v>
       </c>
       <c r="G23" s="55" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="H23" s="55" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="I23" s="55" t="s">
         <v>18</v>
@@ -6923,7 +6923,7 @@
         <v>19</v>
       </c>
       <c r="N23" s="11" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="24" spans="1:14" ht="45" x14ac:dyDescent="0.25">
@@ -6955,10 +6955,10 @@
         <v>0</v>
       </c>
       <c r="J24" s="55" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="K24" s="10" t="s">
-        <v>37</v>
+        <v>72</v>
       </c>
       <c r="L24" s="10">
         <v>0</v>
@@ -6999,10 +6999,10 @@
         <v>0</v>
       </c>
       <c r="J25" s="55" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="K25" s="10" t="s">
-        <v>37</v>
+        <v>72</v>
       </c>
       <c r="L25" s="10">
         <v>0</v>
@@ -7043,10 +7043,10 @@
         <v>0</v>
       </c>
       <c r="J26" s="62" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="K26" s="12" t="s">
-        <v>37</v>
+        <v>72</v>
       </c>
       <c r="L26" s="12">
         <v>0</v>
@@ -7059,13 +7059,13 @@
       </c>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A29" s="46" t="s">
-        <v>47</v>
+      <c r="A29" s="23" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="30" spans="1:14" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A30" s="46" t="s">
-        <v>48</v>
+      <c r="A30" s="23" t="s">
+        <v>92</v>
       </c>
       <c r="B30" s="42"/>
       <c r="C30" s="42"/>
@@ -7073,8 +7073,8 @@
       <c r="E30" s="42"/>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A31" s="46" t="s">
-        <v>49</v>
+      <c r="A31" s="23" t="s">
+        <v>93</v>
       </c>
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
@@ -7090,7 +7090,7 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="46" t="s">
-        <v>71</v>
+        <v>59</v>
       </c>
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
@@ -7099,7 +7099,7 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="46" t="s">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
@@ -7108,7 +7108,7 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="46" t="s">
-        <v>73</v>
+        <v>61</v>
       </c>
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
@@ -7124,7 +7124,7 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="46" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
@@ -7133,7 +7133,7 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="46" t="s">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="B38" s="2"/>
       <c r="C38" s="2"/>
@@ -7149,7 +7149,7 @@
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="46" t="s">
-        <v>55</v>
+        <v>44</v>
       </c>
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
@@ -7158,7 +7158,7 @@
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="46" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>

</xml_diff>